<commit_message>
1. Changed Keycloak port 2. Updated docs
</commit_message>
<xml_diff>
--- a/Docs/SAML_Spring_Keycloak_URLs.xlsx
+++ b/Docs/SAML_Spring_Keycloak_URLs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\SpringBoot_SAML_Keycloak_Demo\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D0884EB-8497-416A-8771-C040A7F970A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E6DAA01-2C14-4F8E-B0C2-090DE0D70F83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,9 +56,6 @@
 http://localhost:9092/saml2/authenticate/keycloak</t>
   </si>
   <si>
-    <t>http://localhost:8081/realms/MySecurityRealm/protocol/saml</t>
-  </si>
-  <si>
     <t>http://localhost:9091/login/saml2/sso/keycloak
 http://localhost:9092/login/saml2/sso/keycloak</t>
   </si>
@@ -67,7 +64,10 @@
 http://localhost:9092/saml2/metadata/keycloak</t>
   </si>
   <si>
-    <t>http://localhost:8081/realms/MySecurityRealm/protocol/saml/descriptor</t>
+    <t>http://localhost:9991/realms/MySecurityRealm/protocol/saml</t>
+  </si>
+  <si>
+    <t>http://localhost:9991/realms/MySecurityRealm/protocol/saml/descriptor</t>
   </si>
 </sst>
 </file>
@@ -396,7 +396,7 @@
     </row>
     <row r="3" spans="1:3" ht="22.65" customHeight="1">
       <c r="A3" s="5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>5</v>
@@ -407,7 +407,7 @@
     </row>
     <row r="4" spans="1:3" ht="34" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>3</v>
@@ -418,7 +418,7 @@
     </row>
     <row r="5" spans="1:3" ht="40" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>3</v>

</xml_diff>